<commit_message>
Last updated on 2026-08-24 10:34:00
</commit_message>
<xml_diff>
--- a/excel2.xlsx
+++ b/excel2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/19a167ca52d16e44/srm-work/teaching/25-26-2/SEC-190/code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/19a167ca52d16e44/srm-work/teaching/git-repos/SEC-190/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A6E6707-F523-F843-B256-EF36AC5D0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{3A6E6707-F523-F843-B256-EF36AC5D0E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{597FB9F6-03D1-A949-BF4B-F54EE08E02E9}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{AB715627-B777-8849-80DF-54FDC253446B}"/>
+    <workbookView xWindow="760" yWindow="820" windowWidth="28040" windowHeight="17180" xr2:uid="{AB715627-B777-8849-80DF-54FDC253446B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -426,26 +426,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>